<commit_message>
refs #16813 - [TECH] Mise à jour jour de l'artefact à partir de Detsala
</commit_message>
<xml_diff>
--- a/xaf-archetype/src/main/resources/archetype-resources/__rootArtifactId__-backserver/src/main/resources/xls/demandes.xlsx
+++ b/xaf-archetype/src/main/resources/archetype-resources/__rootArtifactId__-backserver/src/main/resources/xls/demandes.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java_dev_env\IntelliJWorkspaceBis\derjfer\derjfer-backserver\src\main\resources\xls\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java_dev_env\IntelliJWorkspaceBis\detsala\detsala-backserver\src\main\resources\xls\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -50,7 +50,7 @@
             <charset val="1"/>
           </rPr>
           <t xml:space="preserve">
-jx:area(lastCell="AM3")</t>
+jx:area(lastCell="AP3")</t>
         </r>
       </text>
     </comment>
@@ -74,7 +74,7 @@
             <charset val="1"/>
           </rPr>
           <t xml:space="preserve">
-jx:each(items="demandes" var="demande" lastCell="AM3")</t>
+jx:each(items="demandes" var="demande" lastCell="AP3")</t>
         </r>
       </text>
     </comment>
@@ -83,7 +83,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
   <si>
     <t>Identifiant</t>
   </si>
@@ -97,37 +97,70 @@
     <t>Agent affecté</t>
   </si>
   <si>
+    <t>Langue</t>
+  </si>
+  <si>
+    <t>DEMANDE</t>
+  </si>
+  <si>
     <t>Canal</t>
   </si>
   <si>
-    <t>Langue</t>
+    <t>Courrier ref. interne</t>
+  </si>
+  <si>
+    <t>Courrier date réception</t>
+  </si>
+  <si>
+    <t>FO - INFORMATIONS SUR L'ENTREPRISE D'ORIGINE</t>
+  </si>
+  <si>
+    <t>Pays d'origine du détachement</t>
   </si>
   <si>
     <t>Raison sociale</t>
   </si>
   <si>
-    <t>DEMANDE</t>
-  </si>
-  <si>
-    <t>FO - INFORMATIONS SUR L'ENTREPRISE</t>
-  </si>
-  <si>
-    <t>Avez-vous des délégués du personnel ?</t>
-  </si>
-  <si>
-    <t>Nombre de salariés dans l'entreprise</t>
-  </si>
-  <si>
-    <t>Nom de l'entreprise</t>
-  </si>
-  <si>
-    <t>Courrier ref. interne</t>
-  </si>
-  <si>
-    <t>Courrier date réception</t>
-  </si>
-  <si>
-    <t>FO - INFORMATIONS SUR LA DEROGATION</t>
+    <t>FO - INFORMATIONS SUR LE DETACHEMENT</t>
+  </si>
+  <si>
+    <t>Intervenez-vous dans le cadre d'un chantier ?</t>
+  </si>
+  <si>
+    <t>Nom de l'entreprise d'accueil</t>
+  </si>
+  <si>
+    <t>Nom du chantier</t>
+  </si>
+  <si>
+    <t>DECISION</t>
+  </si>
+  <si>
+    <t>Nombre de salariés détachés</t>
+  </si>
+  <si>
+    <t>Nombre de salariés non détachés</t>
+  </si>
+  <si>
+    <t>Motif</t>
+  </si>
+  <si>
+    <t>${detsalaUtils.convertDateToSring(demande.generic.courrierDateReception)}</t>
+  </si>
+  <si>
+    <t>${demande.contenu.donnee.entreprise.estchantier}</t>
+  </si>
+  <si>
+    <t>${demande.contenu.donnee.entreprise.nomchantier}</t>
+  </si>
+  <si>
+    <t>${demande.contenu.donnee.entreprise.nomentreprise}</t>
+  </si>
+  <si>
+    <t>${demande.contenu.donnee.entrepriseorigine.raisonsociale}</t>
+  </si>
+  <si>
+    <t>${demande.contenu.donnee.entreprise.paysoriginedetachement}</t>
   </si>
   <si>
     <t>${demande.generic.identifiant}</t>
@@ -142,34 +175,22 @@
     <t>${demande.generic.langue}</t>
   </si>
   <si>
-    <t>${demande.contenu.donnee.entreprise.raisonsociale}</t>
-  </si>
-  <si>
-    <t>${derjferUtils.convertDateToSring(demande.generic.dateCreation)}</t>
-  </si>
-  <si>
-    <t>Jours fériés</t>
-  </si>
-  <si>
-    <t>${derjferUtils.getSafeString(demande.generic.agentAffecteNom)}</t>
-  </si>
-  <si>
-    <t>${derjferUtils.convertDateToSring(demande.generic.courrierDateReception)}</t>
-  </si>
-  <si>
-    <t>${demande.contenu.donnee.entreprise.nom}</t>
-  </si>
-  <si>
-    <t>${demande.contenu.donnee.derogation.presencedeleguespersonnel}</t>
-  </si>
-  <si>
-    <t>${demande.contenu.donnee.derogation.nombresalarie}</t>
-  </si>
-  <si>
-    <t>${derjferUtils.getSafeString(demande.generic.courrierRefInterne)}</t>
-  </si>
-  <si>
-    <t>${derjferUtils.convertSelectedJourFeriesTypesToString(demande.contenu.donnee.derogation.joursferies.jourDeL_An, demande.contenu.donnee.derogation.joursferies.sainteDevote,  demande.contenu.donnee.derogation.joursferies.lundiDePaques, demande.contenu.donnee.derogation.joursferies.le1erMai, demande.contenu.donnee.derogation.joursferies.ascension, demande.contenu.donnee.derogation.joursferies.lundiDePentecote, demande.contenu.donnee.derogation.joursferies.feteDieu, demande.contenu.donnee.derogation.joursferies.assomption, demande.contenu.donnee.derogation.joursferies.toussaint, demande.contenu.donnee.derogation.joursferies.feteDuPrince, demande.contenu.donnee.derogation.joursferies.immaculeeConception, demande.contenu.donnee.derogation.joursferies.noel)}</t>
+    <t>${detsalaUtils.convertDateToSring(demande.generic.dateCreation)}</t>
+  </si>
+  <si>
+    <t>${detsalaUtils.getSafeString(demande.generic.agentAffecteNom)}</t>
+  </si>
+  <si>
+    <t>${detsalaUtils.getSafeString(demande.generic.courrierRefInterne)}</t>
+  </si>
+  <si>
+    <t>${demande.generic.motif}</t>
+  </si>
+  <si>
+    <t>${demande.informationsDetachement.nombreSalariesDetaches}</t>
+  </si>
+  <si>
+    <t>${demande.informationsDetachement.nombreSalariesNonDetaches}</t>
   </si>
 </sst>
 </file>
@@ -235,7 +256,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -270,21 +291,6 @@
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -357,8 +363,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -371,46 +375,48 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -422,6 +428,11 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFEDD3EC"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -699,138 +710,181 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N8"/>
+  <dimension ref="A1:P14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.140625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="8.5703125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="15.42578125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="17.7109375" style="1" customWidth="1"/>
-    <col min="5" max="5" width="11.140625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="15.42578125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="20.140625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="24.42578125" style="1" customWidth="1"/>
-    <col min="9" max="9" width="22.42578125" style="2" customWidth="1"/>
-    <col min="10" max="10" width="29.28515625" style="10" customWidth="1"/>
-    <col min="11" max="11" width="26.85546875" style="2" customWidth="1"/>
-    <col min="12" max="12" width="44.85546875" style="6" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="39.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.85546875" style="3"/>
+    <col min="1" max="1" width="17.5703125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="13.140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="13.7109375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="18.140625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="20.85546875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="6.85546875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="19.85546875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="21.85546875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="27.28515625" style="2" customWidth="1"/>
+    <col min="10" max="10" width="33.7109375" style="1" customWidth="1"/>
+    <col min="11" max="11" width="40.5703125" style="2" customWidth="1"/>
+    <col min="12" max="12" width="25.7109375" style="4" customWidth="1"/>
+    <col min="13" max="13" width="27.7109375" style="1" customWidth="1"/>
+    <col min="14" max="14" width="42.85546875" style="3" customWidth="1"/>
+    <col min="15" max="15" width="26.5703125" style="13" customWidth="1"/>
+    <col min="16" max="16" width="29.85546875" style="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="24" t="s">
+    <row r="1" spans="1:16" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="23" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="24"/>
+      <c r="I1" s="23" t="s">
+        <v>9</v>
+      </c>
+      <c r="J1" s="23"/>
+      <c r="K1" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="L1" s="21"/>
+      <c r="M1" s="21"/>
+      <c r="N1" s="20" t="s">
+        <v>16</v>
+      </c>
+      <c r="O1" s="21"/>
+      <c r="P1" s="22"/>
+    </row>
+    <row r="2" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="G2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="22"/>
-      <c r="I1" s="21" t="s">
+      <c r="H2" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="22"/>
-      <c r="K1" s="23" t="s">
+      <c r="I2" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J2" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="K2" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L2" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="M2" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="L1" s="23"/>
-      <c r="M1" s="23"/>
-      <c r="N1" s="4"/>
+      <c r="N2" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="O2" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="P2" s="11" t="s">
+        <v>18</v>
+      </c>
     </row>
-    <row r="2" spans="1:14" s="14" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="7" t="s">
+    <row r="3" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="C3" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="D3" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="E3" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="F3" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="G3" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="L3" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="M3" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="N3" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="O3" s="18" t="s">
+        <v>34</v>
+      </c>
+      <c r="P3" s="19" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="14"/>
+      <c r="B4" s="14"/>
+      <c r="C4" s="14"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="15"/>
+      <c r="F4" s="15"/>
+      <c r="G4" s="17"/>
+      <c r="O4" s="18">
         <v>1</v>
       </c>
-      <c r="C2" s="8" t="s">
-        <v>2</v>
-      </c>
-      <c r="D2" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="E2" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="F2" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="H2" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="I2" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="J2" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="K2" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="L2" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="M2" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="N2" s="13"/>
+      <c r="P4" s="19"/>
     </row>
-    <row r="3" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="15" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3" s="15" t="s">
-        <v>20</v>
-      </c>
-      <c r="C3" s="15" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="E3" s="17" t="s">
-        <v>17</v>
-      </c>
-      <c r="F3" s="17" t="s">
-        <v>18</v>
-      </c>
-      <c r="G3" s="17" t="s">
-        <v>27</v>
-      </c>
-      <c r="H3" s="17" t="s">
-        <v>23</v>
-      </c>
-      <c r="I3" s="18" t="s">
-        <v>24</v>
-      </c>
-      <c r="J3" s="19" t="s">
-        <v>19</v>
-      </c>
-      <c r="K3" s="18" t="s">
-        <v>28</v>
-      </c>
-      <c r="L3" s="20" t="s">
-        <v>25</v>
-      </c>
-      <c r="M3" s="17" t="s">
-        <v>26</v>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="O5" s="13">
+        <f ca="1">SUM(INDIRECT("O4:O" &amp; ROW()-1))</f>
+        <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="E8" s="16"/>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="I14" s="16"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
+    <mergeCell ref="N1:P1"/>
+    <mergeCell ref="A1:H1"/>
     <mergeCell ref="I1:J1"/>
     <mergeCell ref="K1:M1"/>
-    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="8" fitToWidth="0" orientation="landscape" r:id="rId1"/>

</xml_diff>